<commit_message>
Added Student Number column  in Database and Dashboard
</commit_message>
<xml_diff>
--- a/templates/STUDENT INFO REGISTRATION NEW.xlsx
+++ b/templates/STUDENT INFO REGISTRATION NEW.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\csuico\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\192.168.1.118\Webservices\clap.ins\WebCWS\portal-handler\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9252"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9264"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -459,7 +459,7 @@
   <dimension ref="A1:J2"/>
   <sheetFormatPr defaultColWidth="9.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.21875" style="2"/>
     <col min="2" max="2" width="21.44140625" style="4" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.77734375" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="79.77734375" style="3" customWidth="1"/>
@@ -467,7 +467,9 @@
     <col min="6" max="6" width="32.21875" style="4" customWidth="1"/>
     <col min="7" max="7" width="9" style="4" customWidth="1"/>
     <col min="8" max="8" width="11.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="9.21875" style="2"/>
+    <col min="9" max="9" width="9.21875" style="2"/>
+    <col min="10" max="10" width="14.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.21875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">

</xml_diff>